<commit_message>
replotted usgs winter dis
</commit_message>
<xml_diff>
--- a/Output/Tracer-selection/Hungerford_rrmse_table.xlsx
+++ b/Output/Tracer-selection/Hungerford_rrmse_table.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
   <si>
     <t xml:space="preserve">Site</t>
   </si>
@@ -107,37 +107,34 @@
     <t xml:space="preserve">P_mg_L</t>
   </si>
   <si>
-    <t xml:space="preserve"># Dimensions</t>
+    <t xml:space="preserve">Dimensions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Na</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cl</t>
   </si>
   <si>
     <t xml:space="preserve">Mn</t>
   </si>
   <si>
-    <t xml:space="preserve">Ca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Na</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cl</t>
+    <t xml:space="preserve">Cu</t>
   </si>
   <si>
     <t xml:space="preserve">Si</t>
   </si>
   <si>
     <t xml:space="preserve">SO4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P</t>
   </si>
 </sst>
 </file>
@@ -146,13 +143,14 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0.00E+00"/>
+    <numFmt numFmtId="165" formatCode="0.0E+00"/>
   </numFmts>
   <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -212,12 +210,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -347,623 +349,623 @@
   <dimension ref="A1:O13"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="18.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="8" style="0" width="19.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="20.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="20.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="1" width="18.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="8" style="1" width="19.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="20.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="20.49"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="0" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>0.567340561694376</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>0.470558456725787</v>
       </c>
-      <c r="F2" s="0" t="n">
+      <c r="F2" s="1" t="n">
         <v>0.375935995170239</v>
       </c>
-      <c r="G2" s="0" t="n">
+      <c r="G2" s="1" t="n">
         <v>0.363989232647052</v>
       </c>
-      <c r="H2" s="0" t="n">
+      <c r="H2" s="1" t="n">
         <v>0.185191514715682</v>
       </c>
-      <c r="I2" s="0" t="n">
+      <c r="I2" s="1" t="n">
         <v>0.135226975928811</v>
       </c>
-      <c r="J2" s="0" t="n">
+      <c r="J2" s="1" t="n">
         <v>0.134219398142277</v>
       </c>
-      <c r="K2" s="0" t="n">
+      <c r="K2" s="1" t="n">
         <v>0.0184022982927515</v>
       </c>
-      <c r="L2" s="0" t="n">
+      <c r="L2" s="1" t="n">
         <v>0.0183819245772048</v>
       </c>
-      <c r="M2" s="0" t="n">
+      <c r="M2" s="1" t="n">
         <v>0.00880429648929884</v>
       </c>
-      <c r="N2" s="0" t="n">
+      <c r="N2" s="1" t="n">
         <v>0.00316092334321243</v>
       </c>
-      <c r="O2" s="0" t="n">
+      <c r="O2" s="1" t="n">
         <v>9.50566951849143E-016</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>0.122346816263272</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="1" t="n">
         <v>0.0895953600205162</v>
       </c>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="1" t="n">
         <v>0.0869364148273627</v>
       </c>
-      <c r="G3" s="0" t="n">
+      <c r="G3" s="1" t="n">
         <v>0.0863851883128204</v>
       </c>
-      <c r="H3" s="0" t="n">
+      <c r="H3" s="1" t="n">
         <v>0.0835092947150045</v>
       </c>
-      <c r="I3" s="0" t="n">
+      <c r="I3" s="1" t="n">
         <v>0.0828509615255901</v>
       </c>
-      <c r="J3" s="0" t="n">
+      <c r="J3" s="1" t="n">
         <v>0.0420379607138642</v>
       </c>
-      <c r="K3" s="0" t="n">
+      <c r="K3" s="1" t="n">
         <v>0.0237138567345117</v>
       </c>
-      <c r="L3" s="0" t="n">
+      <c r="L3" s="1" t="n">
         <v>0.00452398487914133</v>
       </c>
-      <c r="M3" s="0" t="n">
+      <c r="M3" s="1" t="n">
         <v>0.00237054847501667</v>
       </c>
-      <c r="N3" s="0" t="n">
+      <c r="N3" s="1" t="n">
         <v>0.00194017817443838</v>
       </c>
-      <c r="O3" s="0" t="n">
+      <c r="O3" s="1" t="n">
         <v>3.26417345994841E-016</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>0.0725134178722957</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="1" t="n">
         <v>0.0590918697458474</v>
       </c>
-      <c r="F4" s="0" t="n">
+      <c r="F4" s="1" t="n">
         <v>0.0393682923945916</v>
       </c>
-      <c r="G4" s="0" t="n">
+      <c r="G4" s="1" t="n">
         <v>0.0318177472021038</v>
       </c>
-      <c r="H4" s="0" t="n">
+      <c r="H4" s="1" t="n">
         <v>0.02913796939714</v>
       </c>
-      <c r="I4" s="0" t="n">
+      <c r="I4" s="1" t="n">
         <v>0.0233896098330292</v>
       </c>
-      <c r="J4" s="0" t="n">
+      <c r="J4" s="1" t="n">
         <v>0.0226892953140761</v>
       </c>
-      <c r="K4" s="0" t="n">
+      <c r="K4" s="1" t="n">
         <v>0.0226304762099812</v>
       </c>
-      <c r="L4" s="0" t="n">
+      <c r="L4" s="1" t="n">
         <v>0.0162062989794469</v>
       </c>
-      <c r="M4" s="0" t="n">
+      <c r="M4" s="1" t="n">
         <v>0.0151384613066839</v>
       </c>
-      <c r="N4" s="0" t="n">
+      <c r="N4" s="1" t="n">
         <v>0.00748319005017627</v>
       </c>
-      <c r="O4" s="0" t="n">
+      <c r="O4" s="1" t="n">
         <v>2.1229411530424E-016</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>0.0584650294437207</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="1" t="n">
         <v>0.0480979462634113</v>
       </c>
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="1" t="n">
         <v>0.0398564766545832</v>
       </c>
-      <c r="G5" s="0" t="n">
+      <c r="G5" s="1" t="n">
         <v>0.0330047853434893</v>
       </c>
-      <c r="H5" s="0" t="n">
+      <c r="H5" s="1" t="n">
         <v>0.0319517511911058</v>
       </c>
-      <c r="I5" s="0" t="n">
+      <c r="I5" s="1" t="n">
         <v>0.027865529620127</v>
       </c>
-      <c r="J5" s="0" t="n">
+      <c r="J5" s="1" t="n">
         <v>0.0204304271709252</v>
       </c>
-      <c r="K5" s="0" t="n">
+      <c r="K5" s="1" t="n">
         <v>0.0183130220442796</v>
       </c>
-      <c r="L5" s="0" t="n">
+      <c r="L5" s="1" t="n">
         <v>0.0179191811360371</v>
       </c>
-      <c r="M5" s="0" t="n">
+      <c r="M5" s="1" t="n">
         <v>0.0178058940995022</v>
       </c>
-      <c r="N5" s="0" t="n">
+      <c r="N5" s="1" t="n">
         <v>0.00735633083065833</v>
       </c>
-      <c r="O5" s="0" t="n">
+      <c r="O5" s="1" t="n">
         <v>1.48018393102337E-016</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>0.202864643729082</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="1" t="n">
         <v>0.169630125996657</v>
       </c>
-      <c r="F6" s="0" t="n">
+      <c r="F6" s="1" t="n">
         <v>0.0962808289598957</v>
       </c>
-      <c r="G6" s="0" t="n">
+      <c r="G6" s="1" t="n">
         <v>0.0803873111312819</v>
       </c>
-      <c r="H6" s="0" t="n">
+      <c r="H6" s="1" t="n">
         <v>0.0376356409605384</v>
       </c>
-      <c r="I6" s="0" t="n">
+      <c r="I6" s="1" t="n">
         <v>0.037514792796605</v>
       </c>
-      <c r="J6" s="0" t="n">
+      <c r="J6" s="1" t="n">
         <v>0.0374192383453293</v>
       </c>
-      <c r="K6" s="0" t="n">
+      <c r="K6" s="1" t="n">
         <v>0.0118493299327799</v>
       </c>
-      <c r="L6" s="0" t="n">
+      <c r="L6" s="1" t="n">
         <v>0.0114413432141568</v>
       </c>
-      <c r="M6" s="0" t="n">
+      <c r="M6" s="1" t="n">
         <v>0.0103481035408111</v>
       </c>
-      <c r="N6" s="0" t="n">
+      <c r="N6" s="1" t="n">
         <v>0.00992143995497759</v>
       </c>
-      <c r="O6" s="0" t="n">
+      <c r="O6" s="1" t="n">
         <v>4.06401516267299E-016</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="0" t="n">
+      <c r="C7" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>0.147798781466191</v>
       </c>
-      <c r="E7" s="0" t="n">
+      <c r="E7" s="1" t="n">
         <v>0.139646987425683</v>
       </c>
-      <c r="F7" s="0" t="n">
+      <c r="F7" s="1" t="n">
         <v>0.137734465362995</v>
       </c>
-      <c r="G7" s="0" t="n">
+      <c r="G7" s="1" t="n">
         <v>0.0569297841909225</v>
       </c>
-      <c r="H7" s="0" t="n">
+      <c r="H7" s="1" t="n">
         <v>0.0567754732445868</v>
       </c>
-      <c r="I7" s="0" t="n">
+      <c r="I7" s="1" t="n">
         <v>0.0242015582140622</v>
       </c>
-      <c r="J7" s="0" t="n">
+      <c r="J7" s="1" t="n">
         <v>0.0168551145077108</v>
       </c>
-      <c r="K7" s="0" t="n">
+      <c r="K7" s="1" t="n">
         <v>0.00419439737333718</v>
       </c>
-      <c r="L7" s="0" t="n">
+      <c r="L7" s="1" t="n">
         <v>0.00391967414402359</v>
       </c>
-      <c r="M7" s="0" t="n">
+      <c r="M7" s="1" t="n">
         <v>0.00377095667032239</v>
       </c>
-      <c r="N7" s="0" t="n">
+      <c r="N7" s="1" t="n">
         <v>0.000199172525831773</v>
       </c>
-      <c r="O7" s="0" t="n">
+      <c r="O7" s="1" t="n">
         <v>1.90613646360545E-016</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="0" t="n">
+      <c r="C8" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="1" t="n">
         <v>0.0303405189539692</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E8" s="1" t="n">
         <v>0.0192143744121313</v>
       </c>
-      <c r="F8" s="0" t="n">
+      <c r="F8" s="1" t="n">
         <v>0.0139411518091021</v>
       </c>
-      <c r="G8" s="0" t="n">
+      <c r="G8" s="1" t="n">
         <v>0.0137911273487848</v>
       </c>
-      <c r="H8" s="0" t="n">
+      <c r="H8" s="1" t="n">
         <v>0.00649035164847129</v>
       </c>
-      <c r="I8" s="0" t="n">
+      <c r="I8" s="1" t="n">
         <v>0.00630002260257599</v>
       </c>
-      <c r="J8" s="0" t="n">
+      <c r="J8" s="1" t="n">
         <v>0.00574750163128412</v>
       </c>
-      <c r="K8" s="0" t="n">
+      <c r="K8" s="1" t="n">
         <v>0.00566555300626782</v>
       </c>
-      <c r="L8" s="0" t="n">
+      <c r="L8" s="1" t="n">
         <v>0.00564245490050812</v>
       </c>
-      <c r="M8" s="0" t="n">
+      <c r="M8" s="1" t="n">
         <v>0.000841452789096782</v>
       </c>
-      <c r="N8" s="0" t="n">
+      <c r="N8" s="1" t="n">
         <v>0.000771070929832172</v>
       </c>
-      <c r="O8" s="0" t="n">
+      <c r="O8" s="1" t="n">
         <v>6.60880406574286E-017</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="0" t="n">
+      <c r="C9" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>0.0310043389685702</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="1" t="n">
         <v>0.0249501709411288</v>
       </c>
-      <c r="F9" s="0" t="n">
+      <c r="F9" s="1" t="n">
         <v>0.0170360096673188</v>
       </c>
-      <c r="G9" s="0" t="n">
+      <c r="G9" s="1" t="n">
         <v>0.0165319087519425</v>
       </c>
-      <c r="H9" s="0" t="n">
+      <c r="H9" s="1" t="n">
         <v>0.00650062983990909</v>
       </c>
-      <c r="I9" s="0" t="n">
+      <c r="I9" s="1" t="n">
         <v>0.00554728008424342</v>
       </c>
-      <c r="J9" s="0" t="n">
+      <c r="J9" s="1" t="n">
         <v>0.00551527857769399</v>
       </c>
-      <c r="K9" s="0" t="n">
+      <c r="K9" s="1" t="n">
         <v>0.00511023595156697</v>
       </c>
-      <c r="L9" s="0" t="n">
+      <c r="L9" s="1" t="n">
         <v>0.00501924878274062</v>
       </c>
-      <c r="M9" s="0" t="n">
+      <c r="M9" s="1" t="n">
         <v>0.000674653985987559</v>
       </c>
-      <c r="N9" s="0" t="n">
+      <c r="N9" s="1" t="n">
         <v>0.000572625751880322</v>
       </c>
-      <c r="O9" s="0" t="n">
+      <c r="O9" s="1" t="n">
         <v>8.51409675465264E-017</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="0" t="n">
+      <c r="C10" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D10" s="0" t="n">
+      <c r="D10" s="1" t="n">
         <v>0.255805208404266</v>
       </c>
-      <c r="E10" s="0" t="n">
+      <c r="E10" s="1" t="n">
         <v>0.192516882492842</v>
       </c>
-      <c r="F10" s="0" t="n">
+      <c r="F10" s="1" t="n">
         <v>0.18760733650273</v>
       </c>
-      <c r="G10" s="0" t="n">
+      <c r="G10" s="1" t="n">
         <v>0.145358106130254</v>
       </c>
-      <c r="H10" s="0" t="n">
+      <c r="H10" s="1" t="n">
         <v>0.145281138226597</v>
       </c>
-      <c r="I10" s="0" t="n">
+      <c r="I10" s="1" t="n">
         <v>0.136561292105437</v>
       </c>
-      <c r="J10" s="0" t="n">
+      <c r="J10" s="1" t="n">
         <v>0.0602872415115307</v>
       </c>
-      <c r="K10" s="0" t="n">
+      <c r="K10" s="1" t="n">
         <v>0.0168425074005257</v>
       </c>
-      <c r="L10" s="0" t="n">
+      <c r="L10" s="1" t="n">
         <v>0.0151206127558581</v>
       </c>
-      <c r="M10" s="0" t="n">
+      <c r="M10" s="1" t="n">
         <v>0.0135630626614268</v>
       </c>
-      <c r="N10" s="0" t="n">
+      <c r="N10" s="1" t="n">
         <v>0.0098337267666638</v>
       </c>
-      <c r="O10" s="0" t="n">
+      <c r="O10" s="1" t="n">
         <v>4.03783224338243E-016</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="0" t="n">
+      <c r="C11" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D11" s="0" t="n">
+      <c r="D11" s="1" t="n">
         <v>0.231828601441495</v>
       </c>
-      <c r="E11" s="0" t="n">
+      <c r="E11" s="1" t="n">
         <v>0.0895638217454103</v>
       </c>
-      <c r="F11" s="0" t="n">
+      <c r="F11" s="1" t="n">
         <v>0.0838595613900789</v>
       </c>
-      <c r="G11" s="0" t="n">
+      <c r="G11" s="1" t="n">
         <v>0.0835818248238135</v>
       </c>
-      <c r="H11" s="0" t="n">
+      <c r="H11" s="1" t="n">
         <v>0.047685668476972</v>
       </c>
-      <c r="I11" s="0" t="n">
+      <c r="I11" s="1" t="n">
         <v>0.0473761112251893</v>
       </c>
-      <c r="J11" s="0" t="n">
+      <c r="J11" s="1" t="n">
         <v>0.0369235745055501</v>
       </c>
-      <c r="K11" s="0" t="n">
+      <c r="K11" s="1" t="n">
         <v>0.0353930653450961</v>
       </c>
-      <c r="L11" s="0" t="n">
+      <c r="L11" s="1" t="n">
         <v>0.01332915022989</v>
       </c>
-      <c r="M11" s="0" t="n">
+      <c r="M11" s="1" t="n">
         <v>0.00560924890529826</v>
       </c>
-      <c r="N11" s="0" t="n">
+      <c r="N11" s="1" t="n">
         <v>0.0051487268436586</v>
       </c>
-      <c r="O11" s="0" t="n">
+      <c r="O11" s="1" t="n">
         <v>3.5677463537988E-016</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="0" t="n">
+      <c r="C12" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D12" s="0" t="n">
+      <c r="D12" s="1" t="n">
         <v>0.680979058434798</v>
       </c>
-      <c r="E12" s="0" t="n">
+      <c r="E12" s="1" t="n">
         <v>0.494227403879241</v>
       </c>
-      <c r="F12" s="0" t="n">
+      <c r="F12" s="1" t="n">
         <v>0.494117404709615</v>
       </c>
-      <c r="G12" s="0" t="n">
+      <c r="G12" s="1" t="n">
         <v>0.399062169470221</v>
       </c>
-      <c r="H12" s="0" t="n">
+      <c r="H12" s="1" t="n">
         <v>0.346351909307052</v>
       </c>
-      <c r="I12" s="0" t="n">
+      <c r="I12" s="1" t="n">
         <v>0.183054644378931</v>
       </c>
-      <c r="J12" s="0" t="n">
+      <c r="J12" s="1" t="n">
         <v>0.0769826473772207</v>
       </c>
-      <c r="K12" s="0" t="n">
+      <c r="K12" s="1" t="n">
         <v>0.0768780435341245</v>
       </c>
-      <c r="L12" s="0" t="n">
+      <c r="L12" s="1" t="n">
         <v>0.00967315538659456</v>
       </c>
-      <c r="M12" s="0" t="n">
+      <c r="M12" s="1" t="n">
         <v>0.00889483490550194</v>
       </c>
-      <c r="N12" s="0" t="n">
+      <c r="N12" s="1" t="n">
         <v>0.00805562893351056</v>
       </c>
-      <c r="O12" s="0" t="n">
+      <c r="O12" s="1" t="n">
         <v>1.02518932970207E-015</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="0" t="n">
+      <c r="C13" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D13" s="0" t="n">
+      <c r="D13" s="1" t="n">
         <v>0.599299897508571</v>
       </c>
-      <c r="E13" s="0" t="n">
+      <c r="E13" s="1" t="n">
         <v>0.35706147591222</v>
       </c>
-      <c r="F13" s="0" t="n">
+      <c r="F13" s="1" t="n">
         <v>0.254493638093251</v>
       </c>
-      <c r="G13" s="0" t="n">
+      <c r="G13" s="1" t="n">
         <v>0.144302614740522</v>
       </c>
-      <c r="H13" s="0" t="n">
+      <c r="H13" s="1" t="n">
         <v>0.139377989861727</v>
       </c>
-      <c r="I13" s="0" t="n">
+      <c r="I13" s="1" t="n">
         <v>0.0785685076059155</v>
       </c>
-      <c r="J13" s="0" t="n">
+      <c r="J13" s="1" t="n">
         <v>0.0714604442145064</v>
       </c>
-      <c r="K13" s="0" t="n">
+      <c r="K13" s="1" t="n">
         <v>0.0561162930541843</v>
       </c>
-      <c r="L13" s="0" t="n">
+      <c r="L13" s="1" t="n">
         <v>0.0171732796962474</v>
       </c>
-      <c r="M13" s="0" t="n">
+      <c r="M13" s="1" t="n">
         <v>0.0130821301397303</v>
       </c>
-      <c r="N13" s="0" t="n">
+      <c r="N13" s="1" t="n">
         <v>0.0078630395573469</v>
       </c>
-      <c r="O13" s="0" t="n">
+      <c r="O13" s="1" t="n">
         <v>1.00518651095174E-015</v>
       </c>
     </row>
@@ -983,543 +985,505 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="9.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="9.91"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="L1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="K1" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="L1" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="M1" s="0" t="s">
-        <v>38</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="2" t="n">
+        <v>0.122346816263272</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.0725134178722957</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0.0584650294437207</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.231828601441495</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.202864643729082</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>0.567340561694376</v>
       </c>
-      <c r="C2" s="1" t="n">
-        <v>0.122346816263272</v>
-      </c>
-      <c r="D2" s="1" t="n">
-        <v>0.0725134178722957</v>
-      </c>
-      <c r="E2" s="1" t="n">
-        <v>0.0584650294437207</v>
-      </c>
-      <c r="F2" s="1" t="n">
-        <v>0.202864643729082</v>
-      </c>
-      <c r="G2" s="1" t="n">
+      <c r="H2" s="2" t="n">
+        <v>0.680979058434798</v>
+      </c>
+      <c r="I2" s="2" t="n">
         <v>0.147798781466191</v>
       </c>
-      <c r="H2" s="1" t="n">
+      <c r="J2" s="2" t="n">
+        <v>0.255805208404266</v>
+      </c>
+      <c r="K2" s="2" t="n">
         <v>0.0303405189539692</v>
       </c>
-      <c r="I2" s="1" t="n">
+      <c r="L2" s="2" t="n">
         <v>0.0310043389685702</v>
       </c>
-      <c r="J2" s="1" t="n">
-        <v>0.255805208404266</v>
-      </c>
-      <c r="K2" s="1" t="n">
-        <v>0.231828601441495</v>
-      </c>
-      <c r="L2" s="1" t="n">
-        <v>0.680979058434798</v>
-      </c>
-      <c r="M2" s="1" t="n">
-        <v>0.599299897508571</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="2" t="n">
+        <v>0.0895953600205162</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.0590918697458474</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>0.0480979462634113</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>0.0895638217454103</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0.169630125996657</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>0.470558456725787</v>
       </c>
-      <c r="C3" s="1" t="n">
-        <v>0.0895953600205162</v>
-      </c>
-      <c r="D3" s="1" t="n">
-        <v>0.0590918697458474</v>
-      </c>
-      <c r="E3" s="1" t="n">
-        <v>0.0480979462634113</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>0.169630125996657</v>
-      </c>
-      <c r="G3" s="1" t="n">
+      <c r="H3" s="2" t="n">
+        <v>0.494227403879241</v>
+      </c>
+      <c r="I3" s="2" t="n">
         <v>0.139646987425683</v>
       </c>
-      <c r="H3" s="1" t="n">
+      <c r="J3" s="2" t="n">
+        <v>0.192516882492842</v>
+      </c>
+      <c r="K3" s="2" t="n">
         <v>0.0192143744121313</v>
       </c>
-      <c r="I3" s="1" t="n">
+      <c r="L3" s="2" t="n">
         <v>0.0249501709411288</v>
       </c>
-      <c r="J3" s="1" t="n">
-        <v>0.192516882492842</v>
-      </c>
-      <c r="K3" s="1" t="n">
-        <v>0.0895638217454103</v>
-      </c>
-      <c r="L3" s="1" t="n">
-        <v>0.494227403879241</v>
-      </c>
-      <c r="M3" s="1" t="n">
-        <v>0.35706147591222</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="2" t="n">
+        <v>0.0869364148273627</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0.0393682923945916</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>0.0398564766545832</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.0838595613900789</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0.0962808289598957</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>0.375935995170239</v>
       </c>
-      <c r="C4" s="1" t="n">
-        <v>0.0869364148273627</v>
-      </c>
-      <c r="D4" s="1" t="n">
-        <v>0.0393682923945916</v>
-      </c>
-      <c r="E4" s="1" t="n">
-        <v>0.0398564766545832</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>0.0962808289598957</v>
-      </c>
-      <c r="G4" s="1" t="n">
+      <c r="H4" s="2" t="n">
+        <v>0.494117404709615</v>
+      </c>
+      <c r="I4" s="2" t="n">
         <v>0.137734465362995</v>
       </c>
-      <c r="H4" s="1" t="n">
+      <c r="J4" s="2" t="n">
+        <v>0.18760733650273</v>
+      </c>
+      <c r="K4" s="2" t="n">
         <v>0.0139411518091021</v>
       </c>
-      <c r="I4" s="1" t="n">
+      <c r="L4" s="2" t="n">
         <v>0.0170360096673188</v>
       </c>
-      <c r="J4" s="1" t="n">
-        <v>0.18760733650273</v>
-      </c>
-      <c r="K4" s="1" t="n">
-        <v>0.0838595613900789</v>
-      </c>
-      <c r="L4" s="1" t="n">
-        <v>0.494117404709615</v>
-      </c>
-      <c r="M4" s="1" t="n">
-        <v>0.254493638093251</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="2" t="n">
+        <v>0.0863851883128204</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0.0318177472021038</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>0.0330047853434893</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0.0835818248238135</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.0803873111312819</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>0.363989232647052</v>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>0.0863851883128204</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>0.0318177472021038</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>0.0330047853434893</v>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>0.0803873111312819</v>
-      </c>
-      <c r="G5" s="1" t="n">
+      <c r="H5" s="2" t="n">
+        <v>0.399062169470221</v>
+      </c>
+      <c r="I5" s="2" t="n">
         <v>0.0569297841909225</v>
       </c>
-      <c r="H5" s="1" t="n">
+      <c r="J5" s="2" t="n">
+        <v>0.145358106130254</v>
+      </c>
+      <c r="K5" s="2" t="n">
         <v>0.0137911273487848</v>
       </c>
-      <c r="I5" s="1" t="n">
+      <c r="L5" s="2" t="n">
         <v>0.0165319087519425</v>
       </c>
-      <c r="J5" s="1" t="n">
-        <v>0.145358106130254</v>
-      </c>
-      <c r="K5" s="1" t="n">
-        <v>0.0835818248238135</v>
-      </c>
-      <c r="L5" s="1" t="n">
-        <v>0.399062169470221</v>
-      </c>
-      <c r="M5" s="1" t="n">
-        <v>0.144302614740522</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="n">
+      <c r="B6" s="2" t="n">
+        <v>0.0835092947150045</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.02913796939714</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>0.0319517511911058</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0.047685668476972</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0.0376356409605384</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>0.185191514715682</v>
       </c>
-      <c r="C6" s="1" t="n">
-        <v>0.0835092947150045</v>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>0.02913796939714</v>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>0.0319517511911058</v>
-      </c>
-      <c r="F6" s="1" t="n">
-        <v>0.0376356409605384</v>
-      </c>
-      <c r="G6" s="1" t="n">
+      <c r="H6" s="2" t="n">
+        <v>0.346351909307052</v>
+      </c>
+      <c r="I6" s="2" t="n">
         <v>0.0567754732445868</v>
       </c>
-      <c r="H6" s="1" t="n">
+      <c r="J6" s="2" t="n">
+        <v>0.145281138226597</v>
+      </c>
+      <c r="K6" s="2" t="n">
         <v>0.00649035164847129</v>
       </c>
-      <c r="I6" s="1" t="n">
+      <c r="L6" s="2" t="n">
         <v>0.00650062983990909</v>
       </c>
-      <c r="J6" s="1" t="n">
-        <v>0.145281138226597</v>
-      </c>
-      <c r="K6" s="1" t="n">
-        <v>0.047685668476972</v>
-      </c>
-      <c r="L6" s="1" t="n">
-        <v>0.346351909307052</v>
-      </c>
-      <c r="M6" s="1" t="n">
-        <v>0.139377989861727</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="1" t="n">
+      <c r="B7" s="2" t="n">
+        <v>0.0828509615255901</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.0233896098330292</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0.027865529620127</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0.0473761112251893</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.037514792796605</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>0.135226975928811</v>
       </c>
-      <c r="C7" s="1" t="n">
-        <v>0.0828509615255901</v>
-      </c>
-      <c r="D7" s="1" t="n">
-        <v>0.0233896098330292</v>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>0.027865529620127</v>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>0.037514792796605</v>
-      </c>
-      <c r="G7" s="1" t="n">
+      <c r="H7" s="2" t="n">
+        <v>0.183054644378931</v>
+      </c>
+      <c r="I7" s="2" t="n">
         <v>0.0242015582140622</v>
       </c>
-      <c r="H7" s="1" t="n">
+      <c r="J7" s="2" t="n">
+        <v>0.136561292105437</v>
+      </c>
+      <c r="K7" s="2" t="n">
         <v>0.00630002260257599</v>
       </c>
-      <c r="I7" s="1" t="n">
+      <c r="L7" s="2" t="n">
         <v>0.00554728008424342</v>
       </c>
-      <c r="J7" s="1" t="n">
-        <v>0.136561292105437</v>
-      </c>
-      <c r="K7" s="1" t="n">
-        <v>0.0473761112251893</v>
-      </c>
-      <c r="L7" s="1" t="n">
-        <v>0.183054644378931</v>
-      </c>
-      <c r="M7" s="1" t="n">
-        <v>0.0785685076059155</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="2" t="n">
+        <v>0.0420379607138642</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.0226892953140761</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0.0204304271709252</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0.0369235745055501</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0.0374192383453293</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>0.134219398142277</v>
       </c>
-      <c r="C8" s="1" t="n">
-        <v>0.0420379607138642</v>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>0.0226892953140761</v>
-      </c>
-      <c r="E8" s="1" t="n">
-        <v>0.0204304271709252</v>
-      </c>
-      <c r="F8" s="1" t="n">
-        <v>0.0374192383453293</v>
-      </c>
-      <c r="G8" s="1" t="n">
+      <c r="H8" s="2" t="n">
+        <v>0.0769826473772207</v>
+      </c>
+      <c r="I8" s="2" t="n">
         <v>0.0168551145077108</v>
       </c>
-      <c r="H8" s="1" t="n">
+      <c r="J8" s="2" t="n">
+        <v>0.0602872415115307</v>
+      </c>
+      <c r="K8" s="2" t="n">
         <v>0.00574750163128412</v>
       </c>
-      <c r="I8" s="1" t="n">
+      <c r="L8" s="2" t="n">
         <v>0.00551527857769399</v>
       </c>
-      <c r="J8" s="1" t="n">
-        <v>0.0602872415115307</v>
-      </c>
-      <c r="K8" s="1" t="n">
-        <v>0.0369235745055501</v>
-      </c>
-      <c r="L8" s="1" t="n">
-        <v>0.0769826473772207</v>
-      </c>
-      <c r="M8" s="1" t="n">
-        <v>0.0714604442145064</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="2" t="n">
+        <v>0.0237138567345117</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0.0226304762099812</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>0.0183130220442796</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0.0353930653450961</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0.0118493299327799</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>0.0184022982927515</v>
       </c>
-      <c r="C9" s="1" t="n">
-        <v>0.0237138567345117</v>
-      </c>
-      <c r="D9" s="1" t="n">
-        <v>0.0226304762099812</v>
-      </c>
-      <c r="E9" s="1" t="n">
-        <v>0.0183130220442796</v>
-      </c>
-      <c r="F9" s="1" t="n">
-        <v>0.0118493299327799</v>
-      </c>
-      <c r="G9" s="1" t="n">
+      <c r="H9" s="2" t="n">
+        <v>0.0768780435341245</v>
+      </c>
+      <c r="I9" s="2" t="n">
         <v>0.00419439737333718</v>
       </c>
-      <c r="H9" s="1" t="n">
+      <c r="J9" s="2" t="n">
+        <v>0.0168425074005257</v>
+      </c>
+      <c r="K9" s="2" t="n">
         <v>0.00566555300626782</v>
       </c>
-      <c r="I9" s="1" t="n">
+      <c r="L9" s="2" t="n">
         <v>0.00511023595156697</v>
       </c>
-      <c r="J9" s="1" t="n">
-        <v>0.0168425074005257</v>
-      </c>
-      <c r="K9" s="1" t="n">
-        <v>0.0353930653450961</v>
-      </c>
-      <c r="L9" s="1" t="n">
-        <v>0.0768780435341245</v>
-      </c>
-      <c r="M9" s="1" t="n">
-        <v>0.0561162930541843</v>
-      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="1" t="n">
+      <c r="B10" s="2" t="n">
+        <v>0.00452398487914133</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>0.0162062989794469</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0.0179191811360371</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>0.01332915022989</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0.0114413432141568</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>0.0183819245772048</v>
       </c>
-      <c r="C10" s="1" t="n">
-        <v>0.00452398487914133</v>
-      </c>
-      <c r="D10" s="1" t="n">
-        <v>0.0162062989794469</v>
-      </c>
-      <c r="E10" s="1" t="n">
-        <v>0.0179191811360371</v>
-      </c>
-      <c r="F10" s="1" t="n">
-        <v>0.0114413432141568</v>
-      </c>
-      <c r="G10" s="1" t="n">
+      <c r="H10" s="2" t="n">
+        <v>0.00967315538659456</v>
+      </c>
+      <c r="I10" s="2" t="n">
         <v>0.00391967414402359</v>
       </c>
-      <c r="H10" s="1" t="n">
+      <c r="J10" s="2" t="n">
+        <v>0.0151206127558581</v>
+      </c>
+      <c r="K10" s="2" t="n">
         <v>0.00564245490050812</v>
       </c>
-      <c r="I10" s="1" t="n">
+      <c r="L10" s="2" t="n">
         <v>0.00501924878274062</v>
       </c>
-      <c r="J10" s="1" t="n">
-        <v>0.0151206127558581</v>
-      </c>
-      <c r="K10" s="1" t="n">
-        <v>0.01332915022989</v>
-      </c>
-      <c r="L10" s="1" t="n">
-        <v>0.00967315538659456</v>
-      </c>
-      <c r="M10" s="1" t="n">
-        <v>0.0171732796962474</v>
-      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="1" t="n">
+      <c r="B11" s="2" t="n">
+        <v>0.00237054847501667</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>0.0151384613066839</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>0.0178058940995022</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>0.00560924890529826</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>0.0103481035408111</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>0.00880429648929884</v>
       </c>
-      <c r="C11" s="1" t="n">
-        <v>0.00237054847501667</v>
-      </c>
-      <c r="D11" s="1" t="n">
-        <v>0.0151384613066839</v>
-      </c>
-      <c r="E11" s="1" t="n">
-        <v>0.0178058940995022</v>
-      </c>
-      <c r="F11" s="1" t="n">
-        <v>0.0103481035408111</v>
-      </c>
-      <c r="G11" s="1" t="n">
+      <c r="H11" s="2" t="n">
+        <v>0.00889483490550194</v>
+      </c>
+      <c r="I11" s="2" t="n">
         <v>0.00377095667032239</v>
       </c>
-      <c r="H11" s="1" t="n">
+      <c r="J11" s="2" t="n">
+        <v>0.0135630626614268</v>
+      </c>
+      <c r="K11" s="2" t="n">
         <v>0.000841452789096782</v>
       </c>
-      <c r="I11" s="1" t="n">
+      <c r="L11" s="2" t="n">
         <v>0.000674653985987559</v>
       </c>
-      <c r="J11" s="1" t="n">
-        <v>0.0135630626614268</v>
-      </c>
-      <c r="K11" s="1" t="n">
-        <v>0.00560924890529826</v>
-      </c>
-      <c r="L11" s="1" t="n">
-        <v>0.00889483490550194</v>
-      </c>
-      <c r="M11" s="1" t="n">
-        <v>0.0130821301397303</v>
-      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="1" t="n">
+      <c r="B12" s="2" t="n">
+        <v>0.00194017817443838</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>0.00748319005017627</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>0.00735633083065833</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>0.0051487268436586</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>0.00992143995497759</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>0.00316092334321243</v>
       </c>
-      <c r="C12" s="1" t="n">
-        <v>0.00194017817443838</v>
-      </c>
-      <c r="D12" s="1" t="n">
-        <v>0.00748319005017627</v>
-      </c>
-      <c r="E12" s="1" t="n">
-        <v>0.00735633083065833</v>
-      </c>
-      <c r="F12" s="1" t="n">
-        <v>0.00992143995497759</v>
-      </c>
-      <c r="G12" s="1" t="n">
+      <c r="H12" s="2" t="n">
+        <v>0.00805562893351056</v>
+      </c>
+      <c r="I12" s="2" t="n">
         <v>0.000199172525831773</v>
       </c>
-      <c r="H12" s="1" t="n">
+      <c r="J12" s="2" t="n">
+        <v>0.0098337267666638</v>
+      </c>
+      <c r="K12" s="2" t="n">
         <v>0.000771070929832172</v>
       </c>
-      <c r="I12" s="1" t="n">
+      <c r="L12" s="2" t="n">
         <v>0.000572625751880322</v>
       </c>
-      <c r="J12" s="1" t="n">
-        <v>0.0098337267666638</v>
-      </c>
-      <c r="K12" s="1" t="n">
-        <v>0.0051487268436586</v>
-      </c>
-      <c r="L12" s="1" t="n">
-        <v>0.00805562893351056</v>
-      </c>
-      <c r="M12" s="1" t="n">
-        <v>0.0078630395573469</v>
-      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="1" t="n">
+      <c r="B13" s="2" t="n">
+        <v>3.26417345994841E-016</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>2.1229411530424E-016</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>1.48018393102337E-016</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>3.5677463537988E-016</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>4.06401516267299E-016</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>9.50566951849143E-016</v>
       </c>
-      <c r="C13" s="1" t="n">
-        <v>3.26417345994841E-016</v>
-      </c>
-      <c r="D13" s="1" t="n">
-        <v>2.1229411530424E-016</v>
-      </c>
-      <c r="E13" s="1" t="n">
-        <v>1.48018393102337E-016</v>
-      </c>
-      <c r="F13" s="1" t="n">
-        <v>4.06401516267299E-016</v>
-      </c>
-      <c r="G13" s="1" t="n">
+      <c r="H13" s="2" t="n">
+        <v>1.02518932970207E-015</v>
+      </c>
+      <c r="I13" s="2" t="n">
         <v>1.90613646360545E-016</v>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="J13" s="2" t="n">
+        <v>4.03783224338243E-016</v>
+      </c>
+      <c r="K13" s="2" t="n">
         <v>6.60880406574286E-017</v>
       </c>
-      <c r="I13" s="1" t="n">
+      <c r="L13" s="2" t="n">
         <v>8.51409675465264E-017</v>
-      </c>
-      <c r="J13" s="1" t="n">
-        <v>4.03783224338243E-016</v>
-      </c>
-      <c r="K13" s="1" t="n">
-        <v>3.5677463537988E-016</v>
-      </c>
-      <c r="L13" s="1" t="n">
-        <v>1.02518932970207E-015</v>
-      </c>
-      <c r="M13" s="1" t="n">
-        <v>1.00518651095174E-015</v>
       </c>
     </row>
   </sheetData>

</xml_diff>